<commit_message>
Expose full 69-feature vector in API response
</commit_message>
<xml_diff>
--- a/nba_feature_comparison.xlsx
+++ b/nba_feature_comparison.xlsx
@@ -573,13 +573,13 @@
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>12.8</v>
+        <v>8.1</v>
       </c>
       <c r="C4" s="4" t="n">
-        <v>10.59</v>
+        <v>7.55</v>
       </c>
       <c r="D4" s="4" t="n">
-        <v>-4.49</v>
+        <v>-4.32</v>
       </c>
     </row>
     <row r="5">
@@ -589,10 +589,10 @@
         </is>
       </c>
       <c r="B5" s="4" t="n">
-        <v>0.7871</v>
+        <v>0.6357</v>
       </c>
       <c r="C5" s="4" t="n">
-        <v>0.6797</v>
+        <v>0.6357</v>
       </c>
       <c r="D5" s="4" t="n">
         <v>0.2467</v>
@@ -647,13 +647,13 @@
         </is>
       </c>
       <c r="B10" s="9" t="n">
-        <v>0.041</v>
+        <v>0.042</v>
       </c>
       <c r="C10" s="9" t="n">
         <v>0.042</v>
       </c>
       <c r="D10" s="9" t="n">
-        <v>0.043</v>
+        <v>0.042</v>
       </c>
     </row>
     <row r="11">
@@ -710,14 +710,14 @@
           <t>spread_juice_imbalance</t>
         </is>
       </c>
-      <c r="B14" s="10" t="n">
-        <v>-0.023</v>
+      <c r="B14" s="11" t="n">
+        <v>-0.008999999999999999</v>
       </c>
       <c r="C14" s="10" t="n">
         <v>-0.023</v>
       </c>
-      <c r="D14" s="8" t="n">
-        <v>0</v>
+      <c r="D14" s="9" t="n">
+        <v>0.023</v>
       </c>
     </row>
     <row r="15">
@@ -727,13 +727,13 @@
         </is>
       </c>
       <c r="B15" s="11" t="n">
-        <v>-0.004</v>
+        <v>-0.003</v>
       </c>
       <c r="C15" s="11" t="n">
         <v>-0.003</v>
       </c>
       <c r="D15" s="11" t="n">
-        <v>-0.002</v>
+        <v>-0.003</v>
       </c>
     </row>
     <row r="16">
@@ -922,14 +922,14 @@
           <t>opp_suppression_diff</t>
         </is>
       </c>
-      <c r="B30" s="9" t="n">
-        <v>0.64</v>
-      </c>
-      <c r="C30" s="9" t="n">
-        <v>0.9399999999999999</v>
-      </c>
-      <c r="D30" s="10" t="n">
-        <v>-0.13</v>
+      <c r="B30" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="C30" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="D30" s="8" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="31">

</xml_diff>

<commit_message>
Enrichment: 6 new features + key aliases
</commit_message>
<xml_diff>
--- a/nba_feature_comparison.xlsx
+++ b/nba_feature_comparison.xlsx
@@ -48,12 +48,12 @@
     </font>
     <font>
       <name val="Arial"/>
-      <color rgb="00999999"/>
+      <color rgb="00000000"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Arial"/>
-      <color rgb="00000000"/>
+      <color rgb="00999999"/>
       <sz val="10"/>
     </font>
   </fonts>
@@ -76,12 +76,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E2EFDA"/>
+        <fgColor rgb="00FCE4EC"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FCE4EC"/>
+        <fgColor rgb="00E2EFDA"/>
       </patternFill>
     </fill>
   </fills>
@@ -120,16 +120,16 @@
     <xf numFmtId="0" fontId="4" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -560,10 +560,10 @@
         <v>-15.5</v>
       </c>
       <c r="C3" s="4" t="n">
-        <v>-4.5</v>
+        <v>-3.5</v>
       </c>
       <c r="D3" s="4" t="n">
-        <v>-1.5</v>
+        <v>-2.5</v>
       </c>
     </row>
     <row r="4">
@@ -576,10 +576,10 @@
         <v>8.1</v>
       </c>
       <c r="C4" s="4" t="n">
-        <v>7.55</v>
+        <v>7.65</v>
       </c>
       <c r="D4" s="4" t="n">
-        <v>-4.32</v>
+        <v>-4.37</v>
       </c>
     </row>
     <row r="5">
@@ -592,7 +592,7 @@
         <v>0.6357</v>
       </c>
       <c r="C5" s="4" t="n">
-        <v>0.6357</v>
+        <v>0.5995</v>
       </c>
       <c r="D5" s="4" t="n">
         <v>0.2467</v>
@@ -615,13 +615,13 @@
         </is>
       </c>
       <c r="B8" s="8" t="n">
-        <v>0</v>
+        <v>-15.5</v>
       </c>
       <c r="C8" s="8" t="n">
-        <v>0</v>
+        <v>-3.5</v>
       </c>
       <c r="D8" s="8" t="n">
-        <v>0</v>
+        <v>-2.5</v>
       </c>
     </row>
     <row r="9">
@@ -630,14 +630,14 @@
           <t>implied_prob_home</t>
         </is>
       </c>
-      <c r="B9" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="C9" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="D9" s="8" t="n">
-        <v>0</v>
+      <c r="B9" s="9" t="n">
+        <v>0.931</v>
+      </c>
+      <c r="C9" s="9" t="n">
+        <v>0.6575</v>
+      </c>
+      <c r="D9" s="9" t="n">
+        <v>0.5745</v>
       </c>
     </row>
     <row r="10">
@@ -647,13 +647,13 @@
         </is>
       </c>
       <c r="B10" s="9" t="n">
-        <v>0.042</v>
+        <v>0.0421</v>
       </c>
       <c r="C10" s="9" t="n">
-        <v>0.042</v>
+        <v>0.0421</v>
       </c>
       <c r="D10" s="9" t="n">
-        <v>0.042</v>
+        <v>0.0418</v>
       </c>
     </row>
     <row r="11">
@@ -662,14 +662,14 @@
           <t>home_fav</t>
         </is>
       </c>
-      <c r="B11" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="C11" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="D11" s="8" t="n">
-        <v>0</v>
+      <c r="B11" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="C11" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="D11" s="9" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="12">
@@ -678,14 +678,14 @@
           <t>ou_gap</t>
         </is>
       </c>
-      <c r="B12" s="10" t="n">
-        <v>-4.094</v>
+      <c r="B12" s="8" t="n">
+        <v>-4.0938</v>
       </c>
       <c r="C12" s="9" t="n">
-        <v>6.452</v>
+        <v>6.4517</v>
       </c>
       <c r="D12" s="9" t="n">
-        <v>9.108000000000001</v>
+        <v>9.107900000000001</v>
       </c>
     </row>
     <row r="13">
@@ -694,14 +694,14 @@
           <t>sharp_spread_signal</t>
         </is>
       </c>
-      <c r="B13" s="8" t="n">
+      <c r="B13" s="10" t="n">
         <v>0</v>
       </c>
       <c r="C13" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="D13" s="10" t="n">
-        <v>-3</v>
+        <v>2</v>
+      </c>
+      <c r="D13" s="8" t="n">
+        <v>-4</v>
       </c>
     </row>
     <row r="14">
@@ -711,13 +711,13 @@
         </is>
       </c>
       <c r="B14" s="11" t="n">
-        <v>-0.008999999999999999</v>
-      </c>
-      <c r="C14" s="10" t="n">
-        <v>-0.023</v>
-      </c>
-      <c r="D14" s="9" t="n">
-        <v>0.023</v>
+        <v>-0.0091</v>
+      </c>
+      <c r="C14" s="9" t="n">
+        <v>0.0363</v>
+      </c>
+      <c r="D14" s="8" t="n">
+        <v>-0.0227</v>
       </c>
     </row>
     <row r="15">
@@ -727,13 +727,13 @@
         </is>
       </c>
       <c r="B15" s="11" t="n">
-        <v>-0.003</v>
+        <v>-0.0029</v>
       </c>
       <c r="C15" s="11" t="n">
-        <v>-0.003</v>
+        <v>-0.0029</v>
       </c>
       <c r="D15" s="11" t="n">
-        <v>-0.003</v>
+        <v>-0.0032</v>
       </c>
     </row>
     <row r="16">
@@ -742,13 +742,13 @@
           <t>reverse_line_movement</t>
         </is>
       </c>
-      <c r="B16" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="C16" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="D16" s="8" t="n">
+      <c r="B16" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="C16" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="D16" s="10" t="n">
         <v>0</v>
       </c>
     </row>
@@ -784,14 +784,14 @@
           <t>espn_pregame_wp_pbp</t>
         </is>
       </c>
-      <c r="B20" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="C20" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="D20" s="8" t="n">
-        <v>0</v>
+      <c r="B20" s="9" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="C20" s="9" t="n">
+        <v>0.709</v>
+      </c>
+      <c r="D20" s="9" t="n">
+        <v>0.484</v>
       </c>
     </row>
     <row r="22">
@@ -811,13 +811,13 @@
         </is>
       </c>
       <c r="B23" s="11" t="n">
-        <v>-0.001</v>
+        <v>-0.0005999999999999999</v>
       </c>
       <c r="C23" s="9" t="n">
-        <v>0.014</v>
-      </c>
-      <c r="D23" s="10" t="n">
-        <v>-0.013</v>
+        <v>0.0138</v>
+      </c>
+      <c r="D23" s="8" t="n">
+        <v>-0.0129</v>
       </c>
     </row>
     <row r="24">
@@ -826,14 +826,14 @@
           <t>ftpct_diff</t>
         </is>
       </c>
-      <c r="B24" s="10" t="n">
-        <v>-0.081</v>
-      </c>
-      <c r="C24" s="10" t="n">
-        <v>-0.07000000000000001</v>
+      <c r="B24" s="8" t="n">
+        <v>-0.0813</v>
+      </c>
+      <c r="C24" s="8" t="n">
+        <v>-0.0697</v>
       </c>
       <c r="D24" s="9" t="n">
-        <v>0.047</v>
+        <v>0.0466</v>
       </c>
     </row>
     <row r="25">
@@ -843,13 +843,13 @@
         </is>
       </c>
       <c r="B25" s="11" t="n">
-        <v>0.005</v>
+        <v>0.0054</v>
       </c>
       <c r="C25" s="11" t="n">
-        <v>-0.001</v>
+        <v>-0.0009</v>
       </c>
       <c r="D25" s="11" t="n">
-        <v>0.008</v>
+        <v>0.007900000000000001</v>
       </c>
     </row>
     <row r="26">
@@ -859,13 +859,13 @@
         </is>
       </c>
       <c r="B26" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="C26" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="D26" s="8" t="n">
-        <v>0</v>
+        <v>-0.44</v>
+      </c>
+      <c r="C26" s="9" t="n">
+        <v>0.59</v>
+      </c>
+      <c r="D26" s="9" t="n">
+        <v>1.76</v>
       </c>
     </row>
     <row r="27">
@@ -874,14 +874,14 @@
           <t>ato_ratio_diff</t>
         </is>
       </c>
-      <c r="B27" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="C27" s="8" t="n">
-        <v>0</v>
+      <c r="B27" s="9" t="n">
+        <v>0.14</v>
+      </c>
+      <c r="C27" s="9" t="n">
+        <v>0.04</v>
       </c>
       <c r="D27" s="8" t="n">
-        <v>0</v>
+        <v>-0.3</v>
       </c>
     </row>
     <row r="28">
@@ -891,13 +891,13 @@
         </is>
       </c>
       <c r="B28" s="9" t="n">
-        <v>0.058</v>
+        <v>0.0576</v>
       </c>
       <c r="C28" s="9" t="n">
-        <v>0.089</v>
-      </c>
-      <c r="D28" s="10" t="n">
-        <v>-0.138</v>
+        <v>0.0891</v>
+      </c>
+      <c r="D28" s="8" t="n">
+        <v>-0.1379</v>
       </c>
     </row>
     <row r="29">
@@ -907,13 +907,13 @@
         </is>
       </c>
       <c r="B29" s="9" t="n">
-        <v>0.268</v>
+        <v>0.2675</v>
       </c>
       <c r="C29" s="9" t="n">
-        <v>0.38</v>
-      </c>
-      <c r="D29" s="10" t="n">
-        <v>-0.13</v>
+        <v>0.3798</v>
+      </c>
+      <c r="D29" s="8" t="n">
+        <v>-0.1298</v>
       </c>
     </row>
     <row r="30">
@@ -922,13 +922,13 @@
           <t>opp_suppression_diff</t>
         </is>
       </c>
-      <c r="B30" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="C30" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="D30" s="8" t="n">
+      <c r="B30" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="C30" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="D30" s="10" t="n">
         <v>0</v>
       </c>
     </row>
@@ -938,14 +938,14 @@
           <t>three_value_diff</t>
         </is>
       </c>
-      <c r="B31" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="C31" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="D31" s="8" t="n">
-        <v>0</v>
+      <c r="B31" s="9" t="n">
+        <v>0.0276</v>
+      </c>
+      <c r="C31" s="11" t="n">
+        <v>-0.0077</v>
+      </c>
+      <c r="D31" s="9" t="n">
+        <v>0.0362</v>
       </c>
     </row>
     <row r="32">
@@ -955,13 +955,13 @@
         </is>
       </c>
       <c r="B32" s="11" t="n">
-        <v>0.005</v>
+        <v>0.0054</v>
       </c>
       <c r="C32" s="11" t="n">
-        <v>-0.001</v>
+        <v>-0.0009</v>
       </c>
       <c r="D32" s="11" t="n">
-        <v>0.008</v>
+        <v>0.007900000000000001</v>
       </c>
     </row>
     <row r="33">
@@ -971,13 +971,13 @@
         </is>
       </c>
       <c r="B33" s="9" t="n">
-        <v>0.017</v>
+        <v>0.0171</v>
       </c>
       <c r="C33" s="11" t="n">
-        <v>0.008</v>
+        <v>0.008200000000000001</v>
       </c>
       <c r="D33" s="11" t="n">
-        <v>0.001</v>
+        <v>0.0011</v>
       </c>
     </row>
     <row r="35">
@@ -1002,7 +1002,7 @@
       <c r="C36" s="9" t="n">
         <v>2.18</v>
       </c>
-      <c r="D36" s="10" t="n">
+      <c r="D36" s="8" t="n">
         <v>-6.81</v>
       </c>
     </row>
@@ -1015,7 +1015,7 @@
       <c r="B37" s="9" t="n">
         <v>0.015</v>
       </c>
-      <c r="C37" s="10" t="n">
+      <c r="C37" s="8" t="n">
         <v>-0.018</v>
       </c>
       <c r="D37" s="9" t="n">
@@ -1028,14 +1028,14 @@
           <t>scoring_entropy_diff</t>
         </is>
       </c>
-      <c r="B38" s="8" t="n">
-        <v>0</v>
+      <c r="B38" s="9" t="n">
+        <v>0.015</v>
       </c>
       <c r="C38" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="D38" s="8" t="n">
-        <v>0</v>
+        <v>-0.018</v>
+      </c>
+      <c r="D38" s="9" t="n">
+        <v>0.031</v>
       </c>
     </row>
     <row r="40">
@@ -1060,7 +1060,7 @@
       <c r="C41" s="9" t="n">
         <v>18</v>
       </c>
-      <c r="D41" s="10" t="n">
+      <c r="D41" s="8" t="n">
         <v>-7</v>
       </c>
     </row>
@@ -1070,14 +1070,14 @@
           <t>floor_diff</t>
         </is>
       </c>
-      <c r="B42" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="C42" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="D42" s="8" t="n">
-        <v>0</v>
+      <c r="B42" s="9" t="n">
+        <v>17</v>
+      </c>
+      <c r="C42" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="D42" s="9" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="43">
@@ -1086,14 +1086,14 @@
           <t>consistency_diff</t>
         </is>
       </c>
-      <c r="B43" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="C43" s="8" t="n">
-        <v>0</v>
+      <c r="B43" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="C43" s="9" t="n">
+        <v>13</v>
       </c>
       <c r="D43" s="8" t="n">
-        <v>0</v>
+        <v>-9</v>
       </c>
     </row>
     <row r="44">
@@ -1102,14 +1102,14 @@
           <t>bimodal_diff</t>
         </is>
       </c>
-      <c r="B44" s="8" t="n">
-        <v>0</v>
+      <c r="B44" s="9" t="n">
+        <v>0.903</v>
       </c>
       <c r="C44" s="8" t="n">
-        <v>0</v>
+        <v>-0.096</v>
       </c>
       <c r="D44" s="8" t="n">
-        <v>0</v>
+        <v>-0.408</v>
       </c>
     </row>
     <row r="45">
@@ -1118,13 +1118,13 @@
           <t>score_kurtosis_diff</t>
         </is>
       </c>
-      <c r="B45" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="C45" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="D45" s="8" t="n">
+      <c r="B45" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="C45" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="D45" s="10" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1134,13 +1134,13 @@
           <t>margin_accel_diff</t>
         </is>
       </c>
-      <c r="B46" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="C46" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="D46" s="8" t="n">
+      <c r="B46" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="C46" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="D46" s="10" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1150,13 +1150,13 @@
           <t>momentum_halflife_diff</t>
         </is>
       </c>
-      <c r="B47" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="C47" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="D47" s="8" t="n">
+      <c r="B47" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="C47" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="D47" s="10" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1166,13 +1166,13 @@
           <t>win_aging_diff</t>
         </is>
       </c>
-      <c r="B48" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="C48" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="D48" s="8" t="n">
+      <c r="B48" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="C48" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="D48" s="10" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1182,13 +1182,13 @@
           <t>pyth_residual_diff</t>
         </is>
       </c>
-      <c r="B49" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="C49" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="D49" s="8" t="n">
+      <c r="B49" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="C49" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="D49" s="10" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1198,13 +1198,13 @@
           <t>pyth_luck_diff</t>
         </is>
       </c>
-      <c r="B50" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="C50" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="D50" s="8" t="n">
+      <c r="B50" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="C50" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="D50" s="10" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1214,14 +1214,14 @@
           <t>pace_control_diff</t>
         </is>
       </c>
-      <c r="B51" s="8" t="n">
-        <v>0</v>
+      <c r="B51" s="11" t="n">
+        <v>0.001</v>
       </c>
       <c r="C51" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="D51" s="8" t="n">
-        <v>0</v>
+        <v>-0.0252</v>
+      </c>
+      <c r="D51" s="11" t="n">
+        <v>0.0015</v>
       </c>
     </row>
     <row r="52">
@@ -1230,13 +1230,13 @@
           <t>pace_leverage</t>
         </is>
       </c>
-      <c r="B52" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="C52" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="D52" s="8" t="n">
+      <c r="B52" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="C52" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="D52" s="10" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1246,13 +1246,13 @@
           <t>recovery_diff</t>
         </is>
       </c>
-      <c r="B53" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="C53" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="D53" s="8" t="n">
+      <c r="B53" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="C53" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="D53" s="10" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1263,13 +1263,13 @@
         </is>
       </c>
       <c r="B54" s="9" t="n">
-        <v>0.053</v>
-      </c>
-      <c r="C54" s="10" t="n">
-        <v>-0.015</v>
+        <v>0.0527</v>
+      </c>
+      <c r="C54" s="8" t="n">
+        <v>-0.0151</v>
       </c>
       <c r="D54" s="9" t="n">
-        <v>0.051</v>
+        <v>0.0509</v>
       </c>
     </row>
     <row r="55">
@@ -1278,13 +1278,13 @@
           <t>matchup_ft</t>
         </is>
       </c>
-      <c r="B55" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="C55" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="D55" s="8" t="n">
+      <c r="B55" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="C55" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="D55" s="10" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1294,13 +1294,13 @@
           <t>matchup_orb</t>
         </is>
       </c>
-      <c r="B56" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="C56" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="D56" s="8" t="n">
+      <c r="B56" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="C56" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="D56" s="10" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1320,13 +1320,13 @@
           <t>roll_q4_diff</t>
         </is>
       </c>
-      <c r="B59" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="C59" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="D59" s="8" t="n">
+      <c r="B59" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="C59" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="D59" s="10" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1336,13 +1336,13 @@
           <t>roll_paint_pts_diff</t>
         </is>
       </c>
-      <c r="B60" s="10" t="n">
+      <c r="B60" s="8" t="n">
         <v>-5.4</v>
       </c>
       <c r="C60" s="9" t="n">
         <v>0.2</v>
       </c>
-      <c r="D60" s="10" t="n">
+      <c r="D60" s="8" t="n">
         <v>-8.800000000000001</v>
       </c>
     </row>
@@ -1352,13 +1352,13 @@
           <t>roll_bench_pts_diff</t>
         </is>
       </c>
-      <c r="B61" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="C61" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="D61" s="8" t="n">
+      <c r="B61" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="C61" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="D61" s="10" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1371,10 +1371,10 @@
       <c r="B62" s="9" t="n">
         <v>0.105</v>
       </c>
-      <c r="C62" s="10" t="n">
+      <c r="C62" s="8" t="n">
         <v>-0.019</v>
       </c>
-      <c r="D62" s="10" t="n">
+      <c r="D62" s="8" t="n">
         <v>-0.015</v>
       </c>
     </row>
@@ -1384,13 +1384,13 @@
           <t>roll_three_fg_rate_diff</t>
         </is>
       </c>
-      <c r="B63" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="C63" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="D63" s="8" t="n">
+      <c r="B63" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="C63" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="D63" s="10" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1400,13 +1400,13 @@
           <t>roll_paint_fg_rate_diff</t>
         </is>
       </c>
-      <c r="B64" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="C64" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="D64" s="8" t="n">
+      <c r="B64" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="C64" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="D64" s="10" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1442,13 +1442,13 @@
           <t>b2b_diff</t>
         </is>
       </c>
-      <c r="B68" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="C68" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="D68" s="8" t="n">
+      <c r="B68" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="C68" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="D68" s="10" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1458,13 +1458,13 @@
           <t>home_b2b</t>
         </is>
       </c>
-      <c r="B69" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="C69" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="D69" s="8" t="n">
+      <c r="B69" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="C69" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="D69" s="10" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1474,13 +1474,13 @@
           <t>games_last_14_diff</t>
         </is>
       </c>
-      <c r="B70" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="C70" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="D70" s="8" t="n">
+      <c r="B70" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="C70" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="D70" s="10" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1490,13 +1490,13 @@
           <t>games_diff</t>
         </is>
       </c>
-      <c r="B71" s="10" t="n">
+      <c r="B71" s="8" t="n">
         <v>-1</v>
       </c>
-      <c r="C71" s="10" t="n">
+      <c r="C71" s="8" t="n">
         <v>-1</v>
       </c>
-      <c r="D71" s="10" t="n">
+      <c r="D71" s="8" t="n">
         <v>-1</v>
       </c>
     </row>
@@ -1506,13 +1506,13 @@
           <t>days_since_loss_diff</t>
         </is>
       </c>
-      <c r="B72" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="C72" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="D72" s="8" t="n">
+      <c r="B72" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="C72" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="D72" s="10" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1522,13 +1522,13 @@
           <t>is_early_season</t>
         </is>
       </c>
-      <c r="B73" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="C73" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="D73" s="8" t="n">
+      <c r="B73" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="C73" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="D73" s="10" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1538,13 +1538,13 @@
           <t>is_friday_sat</t>
         </is>
       </c>
-      <c r="B74" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="C74" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="D74" s="8" t="n">
+      <c r="B74" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="C74" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="D74" s="10" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1554,14 +1554,14 @@
           <t>post_allstar</t>
         </is>
       </c>
-      <c r="B75" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="C75" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="D75" s="8" t="n">
-        <v>0</v>
+      <c r="B75" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="C75" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="D75" s="9" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="76">
@@ -1570,14 +1570,14 @@
           <t>post_trade_deadline</t>
         </is>
       </c>
-      <c r="B76" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="C76" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="D76" s="8" t="n">
-        <v>0</v>
+      <c r="B76" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="C76" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="D76" s="9" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="77">
@@ -1586,13 +1586,13 @@
           <t>altitude_factor</t>
         </is>
       </c>
-      <c r="B77" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="C77" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="D77" s="8" t="n">
+      <c r="B77" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="C77" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="D77" s="10" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1628,14 +1628,14 @@
           <t>h2h_avg_margin</t>
         </is>
       </c>
-      <c r="B81" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="C81" s="8" t="n">
-        <v>0</v>
+      <c r="B81" s="9" t="n">
+        <v>37</v>
+      </c>
+      <c r="C81" s="9" t="n">
+        <v>8</v>
       </c>
       <c r="D81" s="8" t="n">
-        <v>0</v>
+        <v>-21.5</v>
       </c>
     </row>
     <row r="82">
@@ -1644,14 +1644,14 @@
           <t>is_revenge_home</t>
         </is>
       </c>
-      <c r="B82" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="C82" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="D82" s="8" t="n">
-        <v>0</v>
+      <c r="B82" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="C82" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="D82" s="9" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="83">
@@ -1660,14 +1660,14 @@
           <t>conference_game</t>
         </is>
       </c>
-      <c r="B83" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="C83" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="D83" s="8" t="n">
-        <v>0</v>
+      <c r="B83" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="C83" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="D83" s="9" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="85">
@@ -1686,13 +1686,13 @@
           <t>after_loss_either</t>
         </is>
       </c>
-      <c r="B86" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="C86" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="D86" s="8" t="n">
+      <c r="B86" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="C86" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="D86" s="10" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1702,10 +1702,10 @@
           <t>away_is_public_team</t>
         </is>
       </c>
-      <c r="B87" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="C87" s="8" t="n">
+      <c r="B87" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="C87" s="10" t="n">
         <v>0</v>
       </c>
       <c r="D87" s="9" t="n">
@@ -1728,14 +1728,14 @@
           <t>elo_diff</t>
         </is>
       </c>
-      <c r="B90" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="C90" s="8" t="n">
-        <v>0</v>
+      <c r="B90" s="9" t="n">
+        <v>233.9</v>
+      </c>
+      <c r="C90" s="9" t="n">
+        <v>166.7</v>
       </c>
       <c r="D90" s="8" t="n">
-        <v>0</v>
+        <v>-1.2</v>
       </c>
     </row>
     <row r="92">
@@ -1754,14 +1754,14 @@
           <t>ref_home_whistle</t>
         </is>
       </c>
-      <c r="B93" s="10" t="n">
+      <c r="B93" s="8" t="n">
         <v>-0.08</v>
       </c>
-      <c r="C93" s="10" t="n">
+      <c r="C93" s="8" t="n">
         <v>-0.186</v>
       </c>
-      <c r="D93" s="10" t="n">
-        <v>-0.3</v>
+      <c r="D93" s="8" t="n">
+        <v>-0.3003</v>
       </c>
     </row>
     <row r="94">
@@ -1770,14 +1770,14 @@
           <t>ref_foul_proxy</t>
         </is>
       </c>
-      <c r="B94" s="10" t="n">
+      <c r="B94" s="8" t="n">
         <v>-0.08</v>
       </c>
-      <c r="C94" s="10" t="n">
+      <c r="C94" s="8" t="n">
         <v>-0.186</v>
       </c>
-      <c r="D94" s="10" t="n">
-        <v>-0.3</v>
+      <c r="D94" s="8" t="n">
+        <v>-0.3003</v>
       </c>
     </row>
     <row r="95">
@@ -1786,13 +1786,13 @@
           <t>ref_ou_bias</t>
         </is>
       </c>
-      <c r="B95" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="C95" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="D95" s="8" t="n">
+      <c r="B95" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="C95" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="D95" s="10" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1802,13 +1802,13 @@
           <t>ref_pace_impact</t>
         </is>
       </c>
-      <c r="B96" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="C96" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="D96" s="8" t="n">
+      <c r="B96" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="C96" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="D96" s="10" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix 9 remaining zero features: rolling PBP fallbacks, schedule derivation, ref approximations
</commit_message>
<xml_diff>
--- a/nba_feature_comparison.xlsx
+++ b/nba_feature_comparison.xlsx
@@ -560,7 +560,7 @@
         <v>-15.5</v>
       </c>
       <c r="C3" s="4" t="n">
-        <v>-3.5</v>
+        <v>-4.5</v>
       </c>
       <c r="D3" s="4" t="n">
         <v>-2.5</v>
@@ -573,13 +573,13 @@
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>8.1</v>
+        <v>8.550000000000001</v>
       </c>
       <c r="C4" s="4" t="n">
-        <v>7.65</v>
+        <v>7.63</v>
       </c>
       <c r="D4" s="4" t="n">
-        <v>-4.37</v>
+        <v>-4.26</v>
       </c>
     </row>
     <row r="5">
@@ -589,10 +589,10 @@
         </is>
       </c>
       <c r="B5" s="4" t="n">
+        <v>0.6797</v>
+      </c>
+      <c r="C5" s="4" t="n">
         <v>0.6357</v>
-      </c>
-      <c r="C5" s="4" t="n">
-        <v>0.5995</v>
       </c>
       <c r="D5" s="4" t="n">
         <v>0.2467</v>
@@ -618,7 +618,7 @@
         <v>-15.5</v>
       </c>
       <c r="C8" s="8" t="n">
-        <v>-3.5</v>
+        <v>-4.5</v>
       </c>
       <c r="D8" s="8" t="n">
         <v>-2.5</v>
@@ -631,7 +631,7 @@
         </is>
       </c>
       <c r="B9" s="9" t="n">
-        <v>0.931</v>
+        <v>0.9231</v>
       </c>
       <c r="C9" s="9" t="n">
         <v>0.6575</v>
@@ -647,7 +647,7 @@
         </is>
       </c>
       <c r="B10" s="9" t="n">
-        <v>0.0421</v>
+        <v>0.0407</v>
       </c>
       <c r="C10" s="9" t="n">
         <v>0.0421</v>
@@ -679,7 +679,7 @@
         </is>
       </c>
       <c r="B12" s="8" t="n">
-        <v>-4.0938</v>
+        <v>-5.0938</v>
       </c>
       <c r="C12" s="9" t="n">
         <v>6.4517</v>
@@ -698,7 +698,7 @@
         <v>0</v>
       </c>
       <c r="C13" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D13" s="8" t="n">
         <v>-4</v>
@@ -713,8 +713,8 @@
       <c r="B14" s="11" t="n">
         <v>-0.0091</v>
       </c>
-      <c r="C14" s="9" t="n">
-        <v>0.0363</v>
+      <c r="C14" s="11" t="n">
+        <v>-0.0091</v>
       </c>
       <c r="D14" s="8" t="n">
         <v>-0.0227</v>
@@ -727,7 +727,7 @@
         </is>
       </c>
       <c r="B15" s="11" t="n">
-        <v>-0.0029</v>
+        <v>-0.0043</v>
       </c>
       <c r="C15" s="11" t="n">
         <v>-0.0029</v>
@@ -922,14 +922,14 @@
           <t>opp_suppression_diff</t>
         </is>
       </c>
-      <c r="B30" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="C30" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="D30" s="10" t="n">
-        <v>0</v>
+      <c r="B30" s="9" t="n">
+        <v>5.18</v>
+      </c>
+      <c r="C30" s="9" t="n">
+        <v>0.31</v>
+      </c>
+      <c r="D30" s="9" t="n">
+        <v>1.17</v>
       </c>
     </row>
     <row r="31">
@@ -1118,14 +1118,14 @@
           <t>score_kurtosis_diff</t>
         </is>
       </c>
-      <c r="B45" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="C45" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="D45" s="10" t="n">
-        <v>0</v>
+      <c r="B45" s="9" t="n">
+        <v>0.903</v>
+      </c>
+      <c r="C45" s="8" t="n">
+        <v>-0.096</v>
+      </c>
+      <c r="D45" s="8" t="n">
+        <v>-0.408</v>
       </c>
     </row>
     <row r="46">
@@ -1134,14 +1134,14 @@
           <t>margin_accel_diff</t>
         </is>
       </c>
-      <c r="B46" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="C46" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="D46" s="10" t="n">
-        <v>0</v>
+      <c r="B46" s="8" t="n">
+        <v>-2.6</v>
+      </c>
+      <c r="C46" s="9" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="D46" s="8" t="n">
+        <v>-10.6</v>
       </c>
     </row>
     <row r="47">
@@ -1150,14 +1150,14 @@
           <t>momentum_halflife_diff</t>
         </is>
       </c>
-      <c r="B47" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="C47" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="D47" s="10" t="n">
-        <v>0</v>
+      <c r="B47" s="9" t="n">
+        <v>9.789999999999999</v>
+      </c>
+      <c r="C47" s="9" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="D47" s="8" t="n">
+        <v>-1.82</v>
       </c>
     </row>
     <row r="48">
@@ -1166,14 +1166,14 @@
           <t>win_aging_diff</t>
         </is>
       </c>
-      <c r="B48" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="C48" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="D48" s="10" t="n">
-        <v>0</v>
+      <c r="B48" s="9" t="n">
+        <v>0.275</v>
+      </c>
+      <c r="C48" s="8" t="n">
+        <v>-0.081</v>
+      </c>
+      <c r="D48" s="9" t="n">
+        <v>0.022</v>
       </c>
     </row>
     <row r="49">
@@ -1182,14 +1182,14 @@
           <t>pyth_residual_diff</t>
         </is>
       </c>
-      <c r="B49" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="C49" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="D49" s="10" t="n">
-        <v>0</v>
+      <c r="B49" s="8" t="n">
+        <v>-0.0277</v>
+      </c>
+      <c r="C49" s="8" t="n">
+        <v>-0.118</v>
+      </c>
+      <c r="D49" s="11" t="n">
+        <v>0.01</v>
       </c>
     </row>
     <row r="50">
@@ -1198,14 +1198,14 @@
           <t>pyth_luck_diff</t>
         </is>
       </c>
-      <c r="B50" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="C50" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="D50" s="10" t="n">
-        <v>0</v>
+      <c r="B50" s="8" t="n">
+        <v>-0.31</v>
+      </c>
+      <c r="C50" s="8" t="n">
+        <v>-1.42</v>
+      </c>
+      <c r="D50" s="9" t="n">
+        <v>0.19</v>
       </c>
     </row>
     <row r="51">
@@ -1230,14 +1230,14 @@
           <t>pace_leverage</t>
         </is>
       </c>
-      <c r="B52" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="C52" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="D52" s="10" t="n">
-        <v>0</v>
+      <c r="B52" s="9" t="n">
+        <v>0.0518</v>
+      </c>
+      <c r="C52" s="9" t="n">
+        <v>0.0361</v>
+      </c>
+      <c r="D52" s="9" t="n">
+        <v>0.0993</v>
       </c>
     </row>
     <row r="53">
@@ -1246,14 +1246,14 @@
           <t>recovery_diff</t>
         </is>
       </c>
-      <c r="B53" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="C53" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="D53" s="10" t="n">
-        <v>0</v>
+      <c r="B53" s="8" t="n">
+        <v>-0.1</v>
+      </c>
+      <c r="C53" s="8" t="n">
+        <v>-0.267</v>
+      </c>
+      <c r="D53" s="8" t="n">
+        <v>-0.25</v>
       </c>
     </row>
     <row r="54">
@@ -1278,14 +1278,14 @@
           <t>matchup_ft</t>
         </is>
       </c>
-      <c r="B55" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="C55" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="D55" s="10" t="n">
-        <v>0</v>
+      <c r="B55" s="9" t="n">
+        <v>0.1054</v>
+      </c>
+      <c r="C55" s="8" t="n">
+        <v>-0.0308</v>
+      </c>
+      <c r="D55" s="8" t="n">
+        <v>-0.0119</v>
       </c>
     </row>
     <row r="56">
@@ -1294,14 +1294,14 @@
           <t>matchup_orb</t>
         </is>
       </c>
-      <c r="B56" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="C56" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="D56" s="10" t="n">
-        <v>0</v>
+      <c r="B56" s="8" t="n">
+        <v>-1.27</v>
+      </c>
+      <c r="C56" s="9" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="D56" s="9" t="n">
+        <v>1.64</v>
       </c>
     </row>
     <row r="58">

</xml_diff>

<commit_message>
Debug components for last 3 zero features
</commit_message>
<xml_diff>
--- a/nba_feature_comparison.xlsx
+++ b/nba_feature_comparison.xlsx
@@ -560,7 +560,7 @@
         <v>-15.5</v>
       </c>
       <c r="C3" s="4" t="n">
-        <v>-4.5</v>
+        <v>-5.5</v>
       </c>
       <c r="D3" s="4" t="n">
         <v>-2.5</v>
@@ -576,7 +576,7 @@
         <v>8.550000000000001</v>
       </c>
       <c r="C4" s="4" t="n">
-        <v>7.63</v>
+        <v>7.66</v>
       </c>
       <c r="D4" s="4" t="n">
         <v>-4.26</v>
@@ -618,7 +618,7 @@
         <v>-15.5</v>
       </c>
       <c r="C8" s="8" t="n">
-        <v>-4.5</v>
+        <v>-5.5</v>
       </c>
       <c r="D8" s="8" t="n">
         <v>-2.5</v>
@@ -634,7 +634,7 @@
         <v>0.9231</v>
       </c>
       <c r="C9" s="9" t="n">
-        <v>0.6575</v>
+        <v>0.6855</v>
       </c>
       <c r="D9" s="9" t="n">
         <v>0.5745</v>
@@ -650,7 +650,7 @@
         <v>0.0407</v>
       </c>
       <c r="C10" s="9" t="n">
-        <v>0.0421</v>
+        <v>0.0427</v>
       </c>
       <c r="D10" s="9" t="n">
         <v>0.0418</v>
@@ -682,7 +682,7 @@
         <v>-5.0938</v>
       </c>
       <c r="C12" s="9" t="n">
-        <v>6.4517</v>
+        <v>7.4517</v>
       </c>
       <c r="D12" s="9" t="n">
         <v>9.107900000000001</v>
@@ -697,8 +697,8 @@
       <c r="B13" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="C13" s="9" t="n">
-        <v>1</v>
+      <c r="C13" s="10" t="n">
+        <v>0</v>
       </c>
       <c r="D13" s="8" t="n">
         <v>-4</v>
@@ -713,8 +713,8 @@
       <c r="B14" s="11" t="n">
         <v>-0.0091</v>
       </c>
-      <c r="C14" s="11" t="n">
-        <v>-0.0091</v>
+      <c r="C14" s="8" t="n">
+        <v>-0.0363</v>
       </c>
       <c r="D14" s="8" t="n">
         <v>-0.0227</v>
@@ -730,7 +730,7 @@
         <v>-0.0043</v>
       </c>
       <c r="C15" s="11" t="n">
-        <v>-0.0029</v>
+        <v>-0.0023</v>
       </c>
       <c r="D15" s="11" t="n">
         <v>-0.0032</v>
@@ -1320,14 +1320,14 @@
           <t>roll_q4_diff</t>
         </is>
       </c>
-      <c r="B59" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="C59" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="D59" s="10" t="n">
-        <v>0</v>
+      <c r="B59" s="8" t="n">
+        <v>-1</v>
+      </c>
+      <c r="C59" s="8" t="n">
+        <v>-2.5</v>
+      </c>
+      <c r="D59" s="8" t="n">
+        <v>-3.6</v>
       </c>
     </row>
     <row r="60">
@@ -1352,14 +1352,14 @@
           <t>roll_bench_pts_diff</t>
         </is>
       </c>
-      <c r="B61" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="C61" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="D61" s="10" t="n">
-        <v>0</v>
+      <c r="B61" s="8" t="n">
+        <v>-3.5</v>
+      </c>
+      <c r="C61" s="9" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="D61" s="9" t="n">
+        <v>3.5</v>
       </c>
     </row>
     <row r="62">
@@ -1384,14 +1384,14 @@
           <t>roll_three_fg_rate_diff</t>
         </is>
       </c>
-      <c r="B63" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="C63" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="D63" s="10" t="n">
-        <v>0</v>
+      <c r="B63" s="9" t="n">
+        <v>0.039</v>
+      </c>
+      <c r="C63" s="11" t="n">
+        <v>-0.008999999999999999</v>
+      </c>
+      <c r="D63" s="9" t="n">
+        <v>0.06</v>
       </c>
     </row>
     <row r="64">
@@ -1686,11 +1686,11 @@
           <t>after_loss_either</t>
         </is>
       </c>
-      <c r="B86" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="C86" s="10" t="n">
-        <v>0</v>
+      <c r="B86" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="C86" s="9" t="n">
+        <v>1</v>
       </c>
       <c r="D86" s="10" t="n">
         <v>0</v>
@@ -1786,14 +1786,14 @@
           <t>ref_ou_bias</t>
         </is>
       </c>
-      <c r="B95" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="C95" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="D95" s="10" t="n">
-        <v>0</v>
+      <c r="B95" s="8" t="n">
+        <v>-0.16</v>
+      </c>
+      <c r="C95" s="8" t="n">
+        <v>-0.372</v>
+      </c>
+      <c r="D95" s="8" t="n">
+        <v>-0.6007</v>
       </c>
     </row>
     <row r="96">
@@ -1802,14 +1802,14 @@
           <t>ref_pace_impact</t>
         </is>
       </c>
-      <c r="B96" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="C96" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="D96" s="10" t="n">
-        <v>0</v>
+      <c r="B96" s="9" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="C96" s="9" t="n">
+        <v>0.093</v>
+      </c>
+      <c r="D96" s="9" t="n">
+        <v>0.1502</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix last 3 zeros: stale days_since_loss, paint_fg_rate derivation
</commit_message>
<xml_diff>
--- a/nba_feature_comparison.xlsx
+++ b/nba_feature_comparison.xlsx
@@ -563,7 +563,7 @@
         <v>-5.5</v>
       </c>
       <c r="D3" s="4" t="n">
-        <v>-2.5</v>
+        <v>-1.5</v>
       </c>
     </row>
     <row r="4">
@@ -579,7 +579,7 @@
         <v>7.66</v>
       </c>
       <c r="D4" s="4" t="n">
-        <v>-4.26</v>
+        <v>-4.16</v>
       </c>
     </row>
     <row r="5">
@@ -621,7 +621,7 @@
         <v>-5.5</v>
       </c>
       <c r="D8" s="8" t="n">
-        <v>-2.5</v>
+        <v>-1.5</v>
       </c>
     </row>
     <row r="9">
@@ -634,7 +634,7 @@
         <v>0.9231</v>
       </c>
       <c r="C9" s="9" t="n">
-        <v>0.6855</v>
+        <v>0.6923</v>
       </c>
       <c r="D9" s="9" t="n">
         <v>0.5745</v>
@@ -650,7 +650,7 @@
         <v>0.0407</v>
       </c>
       <c r="C10" s="9" t="n">
-        <v>0.0427</v>
+        <v>0.0432</v>
       </c>
       <c r="D10" s="9" t="n">
         <v>0.0418</v>
@@ -701,7 +701,7 @@
         <v>0</v>
       </c>
       <c r="D13" s="8" t="n">
-        <v>-4</v>
+        <v>-3</v>
       </c>
     </row>
     <row r="14">
@@ -716,8 +716,8 @@
       <c r="C14" s="8" t="n">
         <v>-0.0363</v>
       </c>
-      <c r="D14" s="8" t="n">
-        <v>-0.0227</v>
+      <c r="D14" s="9" t="n">
+        <v>0.0363</v>
       </c>
     </row>
     <row r="15">
@@ -730,7 +730,7 @@
         <v>-0.0043</v>
       </c>
       <c r="C15" s="11" t="n">
-        <v>-0.0023</v>
+        <v>-0.0018</v>
       </c>
       <c r="D15" s="11" t="n">
         <v>-0.0032</v>

</xml_diff>

<commit_message>
Fix last 2: paint_fg_rate from builder, games_last_14 + days_since_loss from Supabase
</commit_message>
<xml_diff>
--- a/nba_feature_comparison.xlsx
+++ b/nba_feature_comparison.xlsx
@@ -573,7 +573,7 @@
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>8.550000000000001</v>
+        <v>8.56</v>
       </c>
       <c r="C4" s="4" t="n">
         <v>7.66</v>
@@ -679,13 +679,13 @@
         </is>
       </c>
       <c r="B12" s="8" t="n">
-        <v>-5.0938</v>
+        <v>-4.0938</v>
       </c>
       <c r="C12" s="9" t="n">
         <v>7.4517</v>
       </c>
       <c r="D12" s="9" t="n">
-        <v>9.107900000000001</v>
+        <v>10.1079</v>
       </c>
     </row>
     <row r="13">
@@ -1512,8 +1512,8 @@
       <c r="C72" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="D72" s="10" t="n">
-        <v>0</v>
+      <c r="D72" s="8" t="n">
+        <v>-6.6</v>
       </c>
     </row>
     <row r="73">

</xml_diff>

<commit_message>
Banner rework + MLB caps + NBA ML O/U
</commit_message>
<xml_diff>
--- a/nba_feature_comparison.xlsx
+++ b/nba_feature_comparison.xlsx
@@ -560,10 +560,10 @@
         <v>-15.5</v>
       </c>
       <c r="C3" s="4" t="n">
-        <v>-5.5</v>
+        <v>-4.5</v>
       </c>
       <c r="D3" s="4" t="n">
-        <v>-1.5</v>
+        <v>-2.5</v>
       </c>
     </row>
     <row r="4">
@@ -573,13 +573,13 @@
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>8.56</v>
+        <v>8.630000000000001</v>
       </c>
       <c r="C4" s="4" t="n">
-        <v>7.66</v>
+        <v>7.52</v>
       </c>
       <c r="D4" s="4" t="n">
-        <v>-4.16</v>
+        <v>-3.96</v>
       </c>
     </row>
     <row r="5">
@@ -592,7 +592,7 @@
         <v>0.6797</v>
       </c>
       <c r="C5" s="4" t="n">
-        <v>0.6357</v>
+        <v>0.5995</v>
       </c>
       <c r="D5" s="4" t="n">
         <v>0.2467</v>
@@ -618,10 +618,10 @@
         <v>-15.5</v>
       </c>
       <c r="C8" s="8" t="n">
-        <v>-5.5</v>
+        <v>-4.5</v>
       </c>
       <c r="D8" s="8" t="n">
-        <v>-1.5</v>
+        <v>-2.5</v>
       </c>
     </row>
     <row r="9">
@@ -631,13 +631,13 @@
         </is>
       </c>
       <c r="B9" s="9" t="n">
-        <v>0.9231</v>
+        <v>0.931</v>
       </c>
       <c r="C9" s="9" t="n">
         <v>0.6923</v>
       </c>
       <c r="D9" s="9" t="n">
-        <v>0.5745</v>
+        <v>0.5652</v>
       </c>
     </row>
     <row r="10">
@@ -647,13 +647,13 @@
         </is>
       </c>
       <c r="B10" s="9" t="n">
-        <v>0.0407</v>
+        <v>0.0421</v>
       </c>
       <c r="C10" s="9" t="n">
         <v>0.0432</v>
       </c>
       <c r="D10" s="9" t="n">
-        <v>0.0418</v>
+        <v>0.0414</v>
       </c>
     </row>
     <row r="11">
@@ -697,11 +697,11 @@
       <c r="B13" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="C13" s="10" t="n">
-        <v>0</v>
+      <c r="C13" s="9" t="n">
+        <v>1</v>
       </c>
       <c r="D13" s="8" t="n">
-        <v>-3</v>
+        <v>-4</v>
       </c>
     </row>
     <row r="14">
@@ -711,13 +711,13 @@
         </is>
       </c>
       <c r="B14" s="11" t="n">
-        <v>-0.0091</v>
-      </c>
-      <c r="C14" s="8" t="n">
-        <v>-0.0363</v>
-      </c>
-      <c r="D14" s="9" t="n">
-        <v>0.0363</v>
+        <v>0.0091</v>
+      </c>
+      <c r="C14" s="9" t="n">
+        <v>0.0227</v>
+      </c>
+      <c r="D14" s="10" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="15">
@@ -727,13 +727,13 @@
         </is>
       </c>
       <c r="B15" s="11" t="n">
-        <v>-0.0043</v>
+        <v>-0.0029</v>
       </c>
       <c r="C15" s="11" t="n">
         <v>-0.0018</v>
       </c>
       <c r="D15" s="11" t="n">
-        <v>-0.0032</v>
+        <v>-0.0036</v>
       </c>
     </row>
     <row r="16">
@@ -745,8 +745,8 @@
       <c r="B16" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="C16" s="10" t="n">
-        <v>0</v>
+      <c r="C16" s="9" t="n">
+        <v>1</v>
       </c>
       <c r="D16" s="10" t="n">
         <v>0</v>
@@ -769,10 +769,10 @@
         </is>
       </c>
       <c r="B19" s="9" t="n">
-        <v>0.8</v>
+        <v>0.802</v>
       </c>
       <c r="C19" s="9" t="n">
-        <v>0.709</v>
+        <v>0.749</v>
       </c>
       <c r="D19" s="9" t="n">
         <v>0.484</v>
@@ -785,10 +785,10 @@
         </is>
       </c>
       <c r="B20" s="9" t="n">
-        <v>0.8</v>
+        <v>0.802</v>
       </c>
       <c r="C20" s="9" t="n">
-        <v>0.709</v>
+        <v>0.749</v>
       </c>
       <c r="D20" s="9" t="n">
         <v>0.484</v>
@@ -1400,14 +1400,14 @@
           <t>roll_paint_fg_rate_diff</t>
         </is>
       </c>
-      <c r="B64" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="C64" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="D64" s="10" t="n">
-        <v>0</v>
+      <c r="B64" s="8" t="n">
+        <v>-0.0477</v>
+      </c>
+      <c r="C64" s="11" t="n">
+        <v>0.0017</v>
+      </c>
+      <c r="D64" s="8" t="n">
+        <v>-0.07530000000000001</v>
       </c>
     </row>
     <row r="65">
@@ -1477,11 +1477,11 @@
       <c r="B70" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="C70" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="D70" s="10" t="n">
-        <v>0</v>
+      <c r="C70" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="D70" s="8" t="n">
+        <v>-1</v>
       </c>
     </row>
     <row r="71">
@@ -1513,7 +1513,7 @@
         <v>0</v>
       </c>
       <c r="D72" s="8" t="n">
-        <v>-6.6</v>
+        <v>-5</v>
       </c>
     </row>
     <row r="73">

</xml_diff>